<commit_message>
BFTC şablonu: Özet'te 'İdare Yaklaşık Maliyet' adlandırması
İdare miktarıyla hesaplanan tutar teklif değil idarenin yaklaşık maliyetidir.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HeSgjaumyie6wfCEgGCs7w
</commit_message>
<xml_diff>
--- a/ihale-analiz/templates/excel/birim-fiyat.xlsx
+++ b/ihale-analiz/templates/excel/birim-fiyat.xlsx
@@ -633,7 +633,7 @@
       <c r="B4" s="5" t="n"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Teklif tutarı (idare miktarı)</t>
+          <t>İdare Yaklaşık Maliyet</t>
         </is>
       </c>
       <c r="E4" s="6">
@@ -667,7 +667,7 @@
       <c r="B6" s="5" t="n"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Teklif / yaklaşık maliyet</t>
+          <t>İdare YM / açıklanan yaklaşık maliyet</t>
         </is>
       </c>
       <c r="E6" s="7">

</xml_diff>